<commit_message>
Save local changes before pull
</commit_message>
<xml_diff>
--- a/투자내역_투자일지/해외주식_매매내역.xlsx
+++ b/투자내역_투자일지/해외주식_매매내역.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\82108\OneDrive\바탕 화면\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\82108\OneDrive\바탕 화면\investment\investment_strategy\투자내역_투자일지\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7AF04F4-5DFA-4896-BE8A-06C50C09BE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778FEBC9-3F7F-48EC-95F3-F9FE06500758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="23400" xr2:uid="{846F47F3-EAAD-4C96-9254-B3F06D85A831}"/>
+    <workbookView xWindow="31095" yWindow="0" windowWidth="26505" windowHeight="23400" activeTab="1" xr2:uid="{846F47F3-EAAD-4C96-9254-B3F06D85A831}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="ANET_매수전략" sheetId="2" r:id="rId2"/>
+    <sheet name="AMAT" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="128">
   <si>
     <t>종목명</t>
   </si>
@@ -384,6 +386,54 @@
   </si>
   <si>
     <t>2025/05/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">매수 이유 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">통신장비 (라우터, 허브)등의 글로벌 투자수요 증가로 미국 관련 제품의 수출 지속적인 증가 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">매출 예측 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">향후 4분기 연속 매출기록을 갈아치우며 성장할 것으로 예상됨 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">ANET의 매출과 851762와의 통계적 상관관계는 0.91에 달함 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>valuation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>분기 예상매출</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예측 PSR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>현재 PSR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SARIMA  추정 시총</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>주관적 추정 시총</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Target </t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -432,7 +482,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -454,6 +504,15 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -469,6 +528,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1190625</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="그림 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A538D05-8A32-D8B9-6D7C-9B95C11D3487}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1190625" y="847725"/>
+          <a:ext cx="11325225" cy="5619750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="그림 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{010EB6D6-3423-F010-9F95-8A4A855405F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1247775" y="7905750"/>
+          <a:ext cx="11325225" cy="4667250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2787,4 +2939,170 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9971825-A109-4D05-9FEC-BCABB430CA75}">
+  <dimension ref="A2:G71"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.25" customWidth="1"/>
+    <col min="2" max="2" width="14.25" customWidth="1"/>
+    <col min="3" max="3" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>118</v>
+      </c>
+      <c r="B35" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C65" t="s">
+        <v>122</v>
+      </c>
+      <c r="D65" t="s">
+        <v>123</v>
+      </c>
+      <c r="E65" t="s">
+        <v>124</v>
+      </c>
+      <c r="F65" t="s">
+        <v>125</v>
+      </c>
+      <c r="G65" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>121</v>
+      </c>
+      <c r="B66" s="7">
+        <v>45838</v>
+      </c>
+      <c r="C66" s="8">
+        <v>2092.2362119999998</v>
+      </c>
+      <c r="D66" s="8">
+        <v>48.743012</v>
+      </c>
+      <c r="E66">
+        <v>62</v>
+      </c>
+      <c r="F66" s="9">
+        <f>C66*D66</f>
+        <v>101981.89478835053</v>
+      </c>
+      <c r="G66" s="9">
+        <f>C66*E66</f>
+        <v>129718.64514399998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B67" s="7">
+        <v>45930</v>
+      </c>
+      <c r="C67" s="8">
+        <v>2182.2754009999999</v>
+      </c>
+      <c r="D67" s="8">
+        <v>46.946218000000002</v>
+      </c>
+      <c r="E67">
+        <v>62</v>
+      </c>
+      <c r="F67" s="9">
+        <f t="shared" ref="F67:F69" si="0">C67*D67</f>
+        <v>102449.57671138342</v>
+      </c>
+      <c r="G67" s="9">
+        <f t="shared" ref="G67:G69" si="1">C67*E67</f>
+        <v>135301.07486199998</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B68" s="7">
+        <v>46022</v>
+      </c>
+      <c r="C68" s="8">
+        <v>2259.1446369999999</v>
+      </c>
+      <c r="D68" s="8">
+        <v>51.374192999999998</v>
+      </c>
+      <c r="E68">
+        <v>62</v>
+      </c>
+      <c r="F68" s="9">
+        <f t="shared" si="0"/>
+        <v>116061.73259615293</v>
+      </c>
+      <c r="G68" s="9">
+        <f t="shared" si="1"/>
+        <v>140066.96749399998</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B69" s="7">
+        <v>46112</v>
+      </c>
+      <c r="C69" s="8">
+        <v>2317.7815850000002</v>
+      </c>
+      <c r="D69" s="8">
+        <v>51.256346999999998</v>
+      </c>
+      <c r="E69">
+        <v>62</v>
+      </c>
+      <c r="F69" s="9">
+        <f t="shared" si="0"/>
+        <v>118801.01719097</v>
+      </c>
+      <c r="G69" s="9">
+        <f t="shared" si="1"/>
+        <v>143702.45827</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F71" t="s">
+        <v>127</v>
+      </c>
+      <c r="G71">
+        <v>150000</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E49FC8A8-BF85-4896-AF74-7B69626E2163}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>